<commit_message>
Afegit: _ParticipacionsDisponibles, _ParticipacionsUtilitzades, _ParticipacionsOcupades
--HG--
branch : Eliminar PreuParticipacionsOrigen
</commit_message>
<xml_diff>
--- a/Docs/Asian-desglo�.xlsx
+++ b/Docs/Asian-desglo�.xlsx
@@ -882,7 +882,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A8:D21"/>
+  <dimension ref="A1:D14"/>
   <sheetFormatPr defaultRowHeight="14.5"/>
   <cols>
     <col min="1" max="1" width="23.453125" customWidth="1"/>
@@ -890,162 +890,162 @@
     <col min="4" max="4" width="12.08984375" customWidth="1"/>
   </cols>
   <sheetData>
+    <row r="1" spans="1:4">
+      <c r="A1" t="s">
+        <v>11</v>
+      </c>
+      <c r="B1" t="s">
+        <v>4</v>
+      </c>
+      <c r="C1" t="s">
+        <v>7</v>
+      </c>
+      <c r="D1" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4">
+      <c r="A2" t="s">
+        <v>0</v>
+      </c>
+      <c r="B2">
+        <v>27</v>
+      </c>
+      <c r="C2" s="6">
+        <v>58.502000000000002</v>
+      </c>
+      <c r="D2" s="21">
+        <v>999.99</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4">
+      <c r="A3" t="s">
+        <v>14</v>
+      </c>
+      <c r="B3">
+        <v>37</v>
+      </c>
+      <c r="C3" s="6">
+        <v>76.745999999999995</v>
+      </c>
+      <c r="D3" s="21">
+        <v>1000</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4">
+      <c r="A4" t="s">
+        <v>15</v>
+      </c>
+      <c r="B4">
+        <v>2</v>
+      </c>
+      <c r="C4" s="6">
+        <v>-325.52199999999999</v>
+      </c>
+      <c r="D4" s="21">
+        <v>-10271.3550097185</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4">
+      <c r="A5" t="s">
+        <v>15</v>
+      </c>
+      <c r="B5">
+        <v>3</v>
+      </c>
+      <c r="C5" s="6">
+        <v>-24.228999999999999</v>
+      </c>
+      <c r="D5" s="21">
+        <v>-927.65046610283002</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4">
+      <c r="A6" t="s">
+        <v>16</v>
+      </c>
+      <c r="B6">
+        <v>7</v>
+      </c>
+      <c r="C6" s="6">
+        <v>22.006038420699198</v>
+      </c>
+      <c r="D6" s="21">
+        <v>5511.21922614491</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4">
+      <c r="A7" t="s">
+        <v>17</v>
+      </c>
+      <c r="B7">
+        <v>15</v>
+      </c>
+      <c r="C7" s="6">
+        <v>679.64</v>
+      </c>
+      <c r="D7" s="21">
+        <v>15626.31</v>
+      </c>
+    </row>
     <row r="8" spans="1:4">
       <c r="A8" t="s">
-        <v>11</v>
-      </c>
-      <c r="B8" t="s">
-        <v>4</v>
-      </c>
-      <c r="C8" t="s">
-        <v>7</v>
-      </c>
-      <c r="D8" t="s">
-        <v>12</v>
+        <v>18</v>
+      </c>
+      <c r="B8">
+        <v>16</v>
+      </c>
+      <c r="C8" s="6">
+        <v>547.645126</v>
+      </c>
+      <c r="D8" s="21">
+        <v>10000</v>
       </c>
     </row>
     <row r="9" spans="1:4">
       <c r="A9" t="s">
-        <v>0</v>
+        <v>18</v>
       </c>
       <c r="B9">
-        <v>27</v>
+        <v>17</v>
       </c>
       <c r="C9" s="6">
-        <v>58.502000000000002</v>
+        <v>1010.611</v>
       </c>
       <c r="D9" s="21">
-        <v>999.99</v>
+        <v>19999.990000000002</v>
       </c>
     </row>
     <row r="10" spans="1:4">
       <c r="A10" t="s">
-        <v>14</v>
+        <v>19</v>
       </c>
       <c r="B10">
-        <v>37</v>
+        <v>108</v>
       </c>
       <c r="C10" s="6">
-        <v>76.745999999999995</v>
+        <v>0.53749999999999998</v>
       </c>
       <c r="D10" s="21">
         <v>1000</v>
       </c>
     </row>
     <row r="11" spans="1:4">
-      <c r="A11" t="s">
-        <v>15</v>
-      </c>
-      <c r="B11">
-        <v>2</v>
-      </c>
-      <c r="C11" s="6">
-        <v>-325.52199999999999</v>
-      </c>
-      <c r="D11" s="21">
-        <v>-10271.3550097185</v>
-      </c>
-    </row>
-    <row r="12" spans="1:4">
-      <c r="A12" t="s">
-        <v>15</v>
-      </c>
-      <c r="B12">
-        <v>3</v>
-      </c>
-      <c r="C12" s="6">
-        <v>-24.228999999999999</v>
-      </c>
-      <c r="D12" s="21">
-        <v>-927.65046610283002</v>
+      <c r="D11" s="22">
+        <f>SUM(D2:D10)</f>
+        <v>42938.50375032358</v>
       </c>
     </row>
     <row r="13" spans="1:4">
-      <c r="A13" t="s">
-        <v>16</v>
-      </c>
       <c r="B13">
-        <v>7</v>
-      </c>
-      <c r="C13" s="6">
-        <v>22.006038420699198</v>
-      </c>
-      <c r="D13" s="21">
-        <v>5511.21922614491</v>
+        <v>27</v>
       </c>
     </row>
     <row r="14" spans="1:4">
       <c r="A14" t="s">
-        <v>17</v>
-      </c>
-      <c r="B14">
-        <v>15</v>
-      </c>
-      <c r="C14" s="6">
-        <v>679.64</v>
-      </c>
-      <c r="D14" s="21">
-        <v>15626.31</v>
-      </c>
-    </row>
-    <row r="15" spans="1:4">
-      <c r="A15" t="s">
-        <v>18</v>
-      </c>
-      <c r="B15">
-        <v>16</v>
-      </c>
-      <c r="C15" s="6">
-        <v>547.645126</v>
-      </c>
-      <c r="D15" s="21">
-        <v>10000</v>
-      </c>
-    </row>
-    <row r="16" spans="1:4">
-      <c r="A16" t="s">
-        <v>18</v>
-      </c>
-      <c r="B16">
-        <v>17</v>
-      </c>
-      <c r="C16" s="6">
-        <v>1010.611</v>
-      </c>
-      <c r="D16" s="21">
-        <v>19999.990000000002</v>
-      </c>
-    </row>
-    <row r="17" spans="1:4">
-      <c r="A17" t="s">
-        <v>19</v>
-      </c>
-      <c r="B17">
-        <v>108</v>
-      </c>
-      <c r="C17" s="6">
-        <v>0.53749999999999998</v>
-      </c>
-      <c r="D17" s="21">
-        <v>1000</v>
-      </c>
-    </row>
-    <row r="18" spans="1:4">
-      <c r="D18" s="22">
-        <f>SUM(D9:D17)</f>
-        <v>42938.50375032358</v>
-      </c>
-    </row>
-    <row r="20" spans="1:4">
-      <c r="B20">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="21" spans="1:4">
-      <c r="A21" t="s">
         <v>13</v>
       </c>
-      <c r="C21">
+      <c r="C14">
         <v>29</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Nous ajustos i nous documents.
--HG--
branch : Proves PiG
</commit_message>
<xml_diff>
--- a/Docs/Asian-desglo�.xlsx
+++ b/Docs/Asian-desglo�.xlsx
@@ -8,21 +8,22 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Repositoris\C#\_Actiu\InversionsV2\Docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5FBEBD25-61EF-4478-80C4-D84168AA1643}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{91BF12F7-E7B4-41DE-8D12-E6501DE6A20F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="22932" yWindow="0" windowWidth="23256" windowHeight="12576" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="22932" yWindow="0" windowWidth="23256" windowHeight="12576" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Movs" sheetId="3" r:id="rId1"/>
     <sheet name="Sheet1" sheetId="1" r:id="rId2"/>
     <sheet name="Sheet2" sheetId="2" r:id="rId3"/>
+    <sheet name="Orig Vendes Reals" sheetId="4" r:id="rId4"/>
   </sheets>
   <calcPr calcId="191029"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="48" uniqueCount="26">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="84" uniqueCount="49">
   <si>
     <t>1-Optimal Income A-H Grs Acc Hdg EUR</t>
   </si>
@@ -100,16 +101,88 @@
   </si>
   <si>
     <t>PiG Venda</t>
+  </si>
+  <si>
+    <t>Id Orig</t>
+  </si>
+  <si>
+    <t>Nom Fons Orig</t>
+  </si>
+  <si>
+    <t>Data Compra Venda</t>
+  </si>
+  <si>
+    <t>Data Orig Compra</t>
+  </si>
+  <si>
+    <t>PU Orig</t>
+  </si>
+  <si>
+    <t>Parts Orig</t>
+  </si>
+  <si>
+    <t>Parts Ocup.</t>
+  </si>
+  <si>
+    <t>Parts Util</t>
+  </si>
+  <si>
+    <t>Parts Orig Ut</t>
+  </si>
+  <si>
+    <t>Parts en cartera</t>
+  </si>
+  <si>
+    <t>Parts orig en cartera</t>
+  </si>
+  <si>
+    <t>Import Orig venda real</t>
+  </si>
+  <si>
+    <t>Import Orig en cartera</t>
+  </si>
+  <si>
+    <t>Pig Origen venda real</t>
+  </si>
+  <si>
+    <t>PiG Origen en cartera</t>
+  </si>
+  <si>
+    <t>PiG Total</t>
+  </si>
+  <si>
+    <t>CT</t>
+  </si>
+  <si>
+    <t>VT</t>
+  </si>
+  <si>
+    <t>V</t>
+  </si>
+  <si>
+    <t>En cartera</t>
+  </si>
+  <si>
+    <t>C</t>
+  </si>
+  <si>
+    <t>Asian Smaller Companies Fund</t>
+  </si>
+  <si>
+    <t>Biotechnology C USD Acc</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="3">
+  <numFmts count="6">
     <numFmt numFmtId="8" formatCode="#,##0.00\ &quot;€&quot;;[Red]\-#,##0.00\ &quot;€&quot;"/>
     <numFmt numFmtId="164" formatCode="0.000"/>
-    <numFmt numFmtId="169" formatCode="#,##0.000"/>
+    <numFmt numFmtId="165" formatCode="#,##0.000"/>
+    <numFmt numFmtId="166" formatCode="#,##0.000\ &quot;€&quot;;[Red]\-#,##0.000\ &quot;€&quot;"/>
+    <numFmt numFmtId="167" formatCode="#,##0.000\ &quot;€&quot;"/>
+    <numFmt numFmtId="168" formatCode="#,##0.00\ &quot;€&quot;"/>
   </numFmts>
   <fonts count="2" x14ac:knownFonts="1">
     <font>
@@ -128,15 +201,33 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="2">
+  <fills count="5">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.79998168889431442"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF00"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF92D050"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="10">
+  <borders count="11">
     <border>
       <left/>
       <right/>
@@ -243,11 +334,20 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left/>
+      <right style="thick">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="40">
+  <cellXfs count="64">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
@@ -331,7 +431,55 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="169" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="14" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
+    <xf numFmtId="166" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="167" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
+    <xf numFmtId="164" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
+    <xf numFmtId="165" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
+    <xf numFmtId="168" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="14" fontId="0" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="165" fontId="0" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="2" borderId="10" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="14" fontId="0" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
+    <xf numFmtId="167" fontId="0" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="165" fontId="0" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
+    <xf numFmtId="165" fontId="1" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="167" fontId="1" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="164" fontId="1" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="164" fontId="0" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="3" borderId="10" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -742,7 +890,7 @@
         <v>20000.02</v>
       </c>
       <c r="H4" s="4">
-        <f t="shared" ref="H4:H10" si="0">D4+H3</f>
+        <f t="shared" ref="H4:H8" si="0">D4+H3</f>
         <v>2115.5839999999998</v>
       </c>
     </row>
@@ -1374,4 +1522,691 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3596EA1D-6BC1-4561-91C8-DA45EBB01657}">
+  <dimension ref="A1:T14"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="1" max="1" width="4.7265625" customWidth="1"/>
+    <col min="2" max="2" width="5.1796875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="4.90625" customWidth="1"/>
+    <col min="4" max="4" width="11.36328125" customWidth="1"/>
+    <col min="5" max="5" width="11.81640625" customWidth="1"/>
+    <col min="6" max="6" width="11" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="8.81640625" customWidth="1"/>
+    <col min="8" max="8" width="9.1796875" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="9.26953125" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="9.54296875" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="8.81640625" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="9.54296875" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="8.81640625" customWidth="1"/>
+    <col min="14" max="14" width="9.453125" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="10.453125" customWidth="1"/>
+    <col min="16" max="17" width="12.08984375" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="12" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="12.08984375" bestFit="1" customWidth="1"/>
+    <col min="20" max="20" width="11.90625" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:20" ht="31.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A1" s="40" t="s">
+        <v>5</v>
+      </c>
+      <c r="B1" s="41" t="s">
+        <v>4</v>
+      </c>
+      <c r="C1" s="40" t="s">
+        <v>26</v>
+      </c>
+      <c r="D1" s="40" t="s">
+        <v>27</v>
+      </c>
+      <c r="E1" s="42" t="s">
+        <v>28</v>
+      </c>
+      <c r="F1" s="40" t="s">
+        <v>29</v>
+      </c>
+      <c r="G1" s="7" t="s">
+        <v>22</v>
+      </c>
+      <c r="H1" s="7" t="s">
+        <v>30</v>
+      </c>
+      <c r="I1" s="41" t="s">
+        <v>7</v>
+      </c>
+      <c r="J1" s="43" t="s">
+        <v>31</v>
+      </c>
+      <c r="K1" s="40" t="s">
+        <v>32</v>
+      </c>
+      <c r="L1" s="40" t="s">
+        <v>33</v>
+      </c>
+      <c r="M1" s="40" t="s">
+        <v>34</v>
+      </c>
+      <c r="N1" s="40" t="s">
+        <v>35</v>
+      </c>
+      <c r="O1" s="40" t="s">
+        <v>36</v>
+      </c>
+      <c r="P1" s="37" t="s">
+        <v>37</v>
+      </c>
+      <c r="Q1" s="40" t="s">
+        <v>38</v>
+      </c>
+      <c r="R1" s="40" t="s">
+        <v>39</v>
+      </c>
+      <c r="S1" s="40" t="s">
+        <v>40</v>
+      </c>
+      <c r="T1" s="40" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="2" spans="1:20" x14ac:dyDescent="0.35">
+      <c r="A2" s="44" t="s">
+        <v>46</v>
+      </c>
+      <c r="B2" s="44">
+        <v>1</v>
+      </c>
+      <c r="C2" s="44">
+        <v>1</v>
+      </c>
+      <c r="D2" s="44" t="s">
+        <v>47</v>
+      </c>
+      <c r="E2" s="45">
+        <v>41172</v>
+      </c>
+      <c r="F2" s="45">
+        <v>41172</v>
+      </c>
+      <c r="G2" s="46">
+        <v>30.719859180024699</v>
+      </c>
+      <c r="H2" s="47">
+        <v>30.719859180024699</v>
+      </c>
+      <c r="I2" s="48">
+        <v>325.52199999999999</v>
+      </c>
+      <c r="J2" s="55">
+        <v>325.52199999999999</v>
+      </c>
+      <c r="K2" s="48"/>
+      <c r="L2" s="48">
+        <f>L3</f>
+        <v>325.52199999999999</v>
+      </c>
+      <c r="M2" s="48">
+        <f>J2/I2*L2</f>
+        <v>325.52199999999999</v>
+      </c>
+      <c r="N2" s="49">
+        <f>I2-(L2+K2)</f>
+        <v>0</v>
+      </c>
+      <c r="O2" s="49">
+        <f>J2/I2*N2</f>
+        <v>0</v>
+      </c>
+      <c r="P2" s="50">
+        <f>H2*M2</f>
+        <v>9999.99</v>
+      </c>
+      <c r="Q2" s="47">
+        <f>O2*H2</f>
+        <v>0</v>
+      </c>
+      <c r="R2" s="47">
+        <f>SUM(P3)-P2</f>
+        <v>1062.3521872841011</v>
+      </c>
+      <c r="S2" s="47">
+        <f>N2*G$13-Q2</f>
+        <v>0</v>
+      </c>
+      <c r="T2" s="47">
+        <f>R2+S2</f>
+        <v>1062.3521872841011</v>
+      </c>
+    </row>
+    <row r="3" spans="1:20" x14ac:dyDescent="0.35">
+      <c r="A3" s="51" t="s">
+        <v>44</v>
+      </c>
+      <c r="B3" s="52">
+        <v>4</v>
+      </c>
+      <c r="C3" s="51"/>
+      <c r="D3" s="51"/>
+      <c r="E3" s="53">
+        <v>41438</v>
+      </c>
+      <c r="F3" s="56"/>
+      <c r="G3" s="57">
+        <v>33.983393402854801</v>
+      </c>
+      <c r="H3" s="54"/>
+      <c r="I3" s="62">
+        <v>1415.5820000000001</v>
+      </c>
+      <c r="J3" s="63"/>
+      <c r="K3" s="54"/>
+      <c r="L3" s="54">
+        <f>I2</f>
+        <v>325.52199999999999</v>
+      </c>
+      <c r="M3" s="54"/>
+      <c r="N3" s="54"/>
+      <c r="O3" s="54"/>
+      <c r="P3" s="54">
+        <f>L3*G3</f>
+        <v>11062.342187284101</v>
+      </c>
+      <c r="Q3" s="54"/>
+      <c r="R3" s="54"/>
+      <c r="S3" s="54"/>
+      <c r="T3" s="54"/>
+    </row>
+    <row r="4" spans="1:20" x14ac:dyDescent="0.35">
+      <c r="A4" s="44" t="s">
+        <v>46</v>
+      </c>
+      <c r="B4" s="44">
+        <v>2</v>
+      </c>
+      <c r="C4" s="44">
+        <v>2</v>
+      </c>
+      <c r="D4" s="44" t="s">
+        <v>47</v>
+      </c>
+      <c r="E4" s="45">
+        <v>41187</v>
+      </c>
+      <c r="F4" s="45">
+        <v>41187</v>
+      </c>
+      <c r="G4" s="46">
+        <v>31.5534895021488</v>
+      </c>
+      <c r="H4" s="47">
+        <v>31.5534895021488</v>
+      </c>
+      <c r="I4" s="48">
+        <v>1267.6880000000001</v>
+      </c>
+      <c r="J4" s="55">
+        <v>1267.6880000000001</v>
+      </c>
+      <c r="K4" s="48"/>
+      <c r="L4" s="48">
+        <f>SUM(L5:L6)</f>
+        <v>1267.6880000000001</v>
+      </c>
+      <c r="M4" s="48">
+        <f>J4/I4*L4</f>
+        <v>1267.6880000000001</v>
+      </c>
+      <c r="N4" s="49">
+        <f>I4-L4</f>
+        <v>0</v>
+      </c>
+      <c r="O4" s="49">
+        <f>J4/I4*N4</f>
+        <v>0</v>
+      </c>
+      <c r="P4" s="50">
+        <f>H4*M4</f>
+        <v>39999.98000000001</v>
+      </c>
+      <c r="Q4" s="47">
+        <f>O4*H4</f>
+        <v>0</v>
+      </c>
+      <c r="R4" s="47">
+        <f>SUM(P5:P6)-P4</f>
+        <v>3064.9073523338811</v>
+      </c>
+      <c r="S4" s="47">
+        <f>N4*G$13-Q4</f>
+        <v>0</v>
+      </c>
+      <c r="T4" s="47">
+        <f>R4+S4</f>
+        <v>3064.9073523338811</v>
+      </c>
+    </row>
+    <row r="5" spans="1:20" x14ac:dyDescent="0.35">
+      <c r="A5" s="51" t="s">
+        <v>44</v>
+      </c>
+      <c r="B5" s="52">
+        <v>4</v>
+      </c>
+      <c r="C5" s="51"/>
+      <c r="D5" s="51"/>
+      <c r="E5" s="53">
+        <v>41438</v>
+      </c>
+      <c r="F5" s="56"/>
+      <c r="G5" s="57">
+        <v>33.983393402854801</v>
+      </c>
+      <c r="H5" s="54"/>
+      <c r="I5" s="62">
+        <v>1415.5820000000001</v>
+      </c>
+      <c r="J5" s="63"/>
+      <c r="K5" s="54">
+        <f>L3</f>
+        <v>325.52199999999999</v>
+      </c>
+      <c r="L5" s="54">
+        <f>I5-K5</f>
+        <v>1090.0600000000002</v>
+      </c>
+      <c r="M5" s="54"/>
+      <c r="N5" s="54"/>
+      <c r="O5" s="54"/>
+      <c r="P5" s="54">
+        <f>L5*G5</f>
+        <v>37043.937812715914</v>
+      </c>
+      <c r="Q5" s="54"/>
+      <c r="R5" s="54"/>
+      <c r="S5" s="54"/>
+      <c r="T5" s="54"/>
+    </row>
+    <row r="6" spans="1:20" x14ac:dyDescent="0.35">
+      <c r="A6" s="51" t="s">
+        <v>44</v>
+      </c>
+      <c r="B6" s="52">
+        <v>5</v>
+      </c>
+      <c r="C6" s="51"/>
+      <c r="D6" s="51"/>
+      <c r="E6" s="53">
+        <v>41492.000694444447</v>
+      </c>
+      <c r="F6" s="56"/>
+      <c r="G6" s="57">
+        <v>33.896398876404497</v>
+      </c>
+      <c r="H6" s="54"/>
+      <c r="I6" s="62">
+        <v>178</v>
+      </c>
+      <c r="J6" s="63"/>
+      <c r="K6" s="54"/>
+      <c r="L6" s="54">
+        <f>I4-L5</f>
+        <v>177.62799999999993</v>
+      </c>
+      <c r="M6" s="54"/>
+      <c r="N6" s="54"/>
+      <c r="O6" s="54"/>
+      <c r="P6" s="54">
+        <f>L6*G6</f>
+        <v>6020.9495396179755</v>
+      </c>
+      <c r="Q6" s="54"/>
+      <c r="R6" s="54"/>
+      <c r="S6" s="54"/>
+      <c r="T6" s="54"/>
+    </row>
+    <row r="7" spans="1:20" x14ac:dyDescent="0.35">
+      <c r="A7" s="44" t="s">
+        <v>46</v>
+      </c>
+      <c r="B7" s="44">
+        <v>3</v>
+      </c>
+      <c r="C7" s="44">
+        <v>3</v>
+      </c>
+      <c r="D7" s="44" t="s">
+        <v>47</v>
+      </c>
+      <c r="E7" s="45">
+        <v>41410</v>
+      </c>
+      <c r="F7" s="45">
+        <v>41410</v>
+      </c>
+      <c r="G7" s="46">
+        <v>38.286783032846202</v>
+      </c>
+      <c r="H7" s="47">
+        <v>38.286783032846202</v>
+      </c>
+      <c r="I7" s="48">
+        <v>522.37400000000002</v>
+      </c>
+      <c r="J7" s="55">
+        <v>522.37400000000002</v>
+      </c>
+      <c r="K7" s="48"/>
+      <c r="L7" s="48">
+        <f>SUM(L8:L9)</f>
+        <v>522.37400000000002</v>
+      </c>
+      <c r="M7" s="48">
+        <f>J7/I7*L7</f>
+        <v>522.37400000000002</v>
+      </c>
+      <c r="N7" s="49">
+        <f>I7-L7</f>
+        <v>0</v>
+      </c>
+      <c r="O7" s="49">
+        <f>J7/I7*N7</f>
+        <v>0</v>
+      </c>
+      <c r="P7" s="50">
+        <f>H7*M7</f>
+        <v>20000.020000000004</v>
+      </c>
+      <c r="Q7" s="47">
+        <f>O7*H7</f>
+        <v>0</v>
+      </c>
+      <c r="R7" s="47">
+        <f>SUM(P8:P9)-P7</f>
+        <v>-3037.8505396179899</v>
+      </c>
+      <c r="S7" s="47">
+        <f>N7*G$13-Q7</f>
+        <v>0</v>
+      </c>
+      <c r="T7" s="47">
+        <f>R7+S7</f>
+        <v>-3037.8505396179899</v>
+      </c>
+    </row>
+    <row r="8" spans="1:20" x14ac:dyDescent="0.35">
+      <c r="A8" s="51" t="s">
+        <v>44</v>
+      </c>
+      <c r="B8" s="52">
+        <v>5</v>
+      </c>
+      <c r="C8" s="51"/>
+      <c r="D8" s="51"/>
+      <c r="E8" s="53">
+        <v>41492.000694444447</v>
+      </c>
+      <c r="F8" s="56"/>
+      <c r="G8" s="57">
+        <v>33.896398876404497</v>
+      </c>
+      <c r="H8" s="54"/>
+      <c r="I8" s="62">
+        <v>178</v>
+      </c>
+      <c r="J8" s="63"/>
+      <c r="K8" s="54">
+        <f>L6</f>
+        <v>177.62799999999993</v>
+      </c>
+      <c r="L8" s="54">
+        <f>I8-K8</f>
+        <v>0.37200000000007094</v>
+      </c>
+      <c r="M8" s="54"/>
+      <c r="N8" s="54"/>
+      <c r="O8" s="54"/>
+      <c r="P8" s="54">
+        <f>L8*G8</f>
+        <v>12.609460382024878</v>
+      </c>
+      <c r="Q8" s="54"/>
+      <c r="R8" s="54"/>
+      <c r="S8" s="54"/>
+      <c r="T8" s="54"/>
+    </row>
+    <row r="9" spans="1:20" x14ac:dyDescent="0.35">
+      <c r="A9" s="51" t="s">
+        <v>44</v>
+      </c>
+      <c r="B9" s="52">
+        <v>6</v>
+      </c>
+      <c r="C9" s="51"/>
+      <c r="D9" s="51"/>
+      <c r="E9" s="53">
+        <v>41506</v>
+      </c>
+      <c r="F9" s="56"/>
+      <c r="G9" s="57">
+        <v>32.470297048670297</v>
+      </c>
+      <c r="H9" s="54"/>
+      <c r="I9" s="62">
+        <v>522.00199999999995</v>
+      </c>
+      <c r="J9" s="63"/>
+      <c r="K9" s="54"/>
+      <c r="L9" s="54">
+        <f>I7-L8</f>
+        <v>522.00199999999995</v>
+      </c>
+      <c r="M9" s="54"/>
+      <c r="N9" s="54"/>
+      <c r="O9" s="54"/>
+      <c r="P9" s="54">
+        <f>L9*G9</f>
+        <v>16949.55999999999</v>
+      </c>
+      <c r="Q9" s="54"/>
+      <c r="R9" s="54"/>
+      <c r="S9" s="54"/>
+      <c r="T9" s="54"/>
+    </row>
+    <row r="10" spans="1:20" x14ac:dyDescent="0.35">
+      <c r="A10" s="44" t="s">
+        <v>42</v>
+      </c>
+      <c r="B10" s="44">
+        <v>41</v>
+      </c>
+      <c r="C10" s="44">
+        <v>7</v>
+      </c>
+      <c r="D10" s="44" t="s">
+        <v>48</v>
+      </c>
+      <c r="E10" s="45">
+        <v>42047.000011574077</v>
+      </c>
+      <c r="F10" s="45">
+        <v>41492.001388888886</v>
+      </c>
+      <c r="G10" s="46">
+        <v>39.4291363665061</v>
+      </c>
+      <c r="H10" s="47">
+        <v>250.44122530300501</v>
+      </c>
+      <c r="I10" s="48">
+        <v>174.22900000000001</v>
+      </c>
+      <c r="J10" s="55">
+        <v>15</v>
+      </c>
+      <c r="K10" s="48"/>
+      <c r="L10" s="48">
+        <f>SUM(L11:L12)</f>
+        <v>174.22899999999998</v>
+      </c>
+      <c r="M10" s="48">
+        <f>J10/I10*L10</f>
+        <v>14.999999999999998</v>
+      </c>
+      <c r="N10" s="49">
+        <f>I10-L10</f>
+        <v>0</v>
+      </c>
+      <c r="O10" s="49">
+        <f>J10/I10*N10</f>
+        <v>0</v>
+      </c>
+      <c r="P10" s="50">
+        <f>H10*M10</f>
+        <v>3756.6183795450747</v>
+      </c>
+      <c r="Q10" s="47">
+        <f>O10*H10</f>
+        <v>0</v>
+      </c>
+      <c r="R10" s="47">
+        <f>SUM(P11:P12)-P10</f>
+        <v>3210.1466479069309</v>
+      </c>
+      <c r="S10" s="47">
+        <f>N10*G$13-Q10</f>
+        <v>0</v>
+      </c>
+      <c r="T10" s="47">
+        <f>R10+S10</f>
+        <v>3210.1466479069309</v>
+      </c>
+    </row>
+    <row r="11" spans="1:20" x14ac:dyDescent="0.35">
+      <c r="A11" s="51" t="s">
+        <v>43</v>
+      </c>
+      <c r="B11" s="52">
+        <v>95</v>
+      </c>
+      <c r="C11" s="51"/>
+      <c r="D11" s="51"/>
+      <c r="E11" s="53">
+        <v>42207.759375000001</v>
+      </c>
+      <c r="F11" s="51"/>
+      <c r="G11" s="57">
+        <v>39.577666666666701</v>
+      </c>
+      <c r="H11" s="54"/>
+      <c r="I11" s="62">
+        <v>150</v>
+      </c>
+      <c r="J11" s="63"/>
+      <c r="K11" s="54"/>
+      <c r="L11" s="54">
+        <f>I11</f>
+        <v>150</v>
+      </c>
+      <c r="M11" s="54"/>
+      <c r="N11" s="54"/>
+      <c r="O11" s="54"/>
+      <c r="P11" s="54">
+        <f>L11*G11</f>
+        <v>5936.6500000000051</v>
+      </c>
+      <c r="Q11" s="54"/>
+      <c r="R11" s="54"/>
+      <c r="S11" s="54"/>
+      <c r="T11" s="54"/>
+    </row>
+    <row r="12" spans="1:20" x14ac:dyDescent="0.35">
+      <c r="A12" s="51" t="s">
+        <v>44</v>
+      </c>
+      <c r="B12" s="52">
+        <v>187</v>
+      </c>
+      <c r="C12" s="51"/>
+      <c r="D12" s="51"/>
+      <c r="E12" s="53">
+        <v>44176.609131944446</v>
+      </c>
+      <c r="F12" s="51"/>
+      <c r="G12" s="57">
+        <v>42.515788000000001</v>
+      </c>
+      <c r="H12" s="54"/>
+      <c r="I12" s="62">
+        <v>24.228999999999999</v>
+      </c>
+      <c r="J12" s="63"/>
+      <c r="K12" s="54"/>
+      <c r="L12" s="54">
+        <f>I12</f>
+        <v>24.228999999999999</v>
+      </c>
+      <c r="M12" s="54"/>
+      <c r="N12" s="54"/>
+      <c r="O12" s="54"/>
+      <c r="P12" s="54">
+        <f>L12*G12</f>
+        <v>1030.115027452</v>
+      </c>
+      <c r="Q12" s="54"/>
+      <c r="R12" s="54"/>
+      <c r="S12" s="54"/>
+      <c r="T12" s="54"/>
+    </row>
+    <row r="13" spans="1:20" s="39" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="A13" s="58"/>
+      <c r="B13" s="58"/>
+      <c r="C13" s="58"/>
+      <c r="D13" s="59" t="s">
+        <v>45</v>
+      </c>
+      <c r="E13" s="58"/>
+      <c r="F13" s="58"/>
+      <c r="G13" s="60">
+        <v>0</v>
+      </c>
+      <c r="H13" s="58"/>
+      <c r="I13" s="58"/>
+      <c r="J13" s="58"/>
+      <c r="K13" s="58"/>
+      <c r="L13" s="58"/>
+      <c r="M13" s="58"/>
+      <c r="N13" s="61">
+        <f>SUM(N2:N12)</f>
+        <v>0</v>
+      </c>
+      <c r="O13" s="61"/>
+      <c r="P13" s="58"/>
+      <c r="Q13" s="60">
+        <f>SUM(Q2:Q12)</f>
+        <v>0</v>
+      </c>
+      <c r="R13" s="60">
+        <f>SUM(R2:R12)</f>
+        <v>4299.5556479069237</v>
+      </c>
+      <c r="S13" s="60">
+        <f>SUM(S2:S12)</f>
+        <v>0</v>
+      </c>
+      <c r="T13" s="60">
+        <f>SUM(T2:T12)</f>
+        <v>4299.5556479069237</v>
+      </c>
+    </row>
+    <row r="14" spans="1:20" x14ac:dyDescent="0.35">
+      <c r="J14" s="39"/>
+      <c r="K14" s="39"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="0" verticalDpi="0" r:id="rId1"/>
+</worksheet>
 </file>
</xml_diff>